<commit_message>
fix: restore axis titles with manual plot area layout to prevent label overlap
Re-add x_title (Owner/Sprint) and y_title (Hours) to bar charts.
Use ManualLayout to reserve 14% left margin and 16% bottom margin so
axis titles don't overlap with tick labels.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/output/ESTIMATE_dashboard.xlsx
+++ b/data/output/ESTIMATE_dashboard.xlsx
@@ -506,7 +506,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -654,7 +654,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -802,7 +802,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -950,7 +950,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1098,7 +1098,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1246,7 +1246,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1394,7 +1394,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1542,7 +1542,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1690,7 +1690,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1838,7 +1838,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -1986,7 +1986,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -2134,7 +2134,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -2282,7 +2282,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>
@@ -2430,7 +2430,7 @@
                   <a:defRPr/>
                 </a:pPr>
                 <a:r>
-                  <a:t>Planned For</a:t>
+                  <a:t>Sprint</a:t>
                 </a:r>
               </a:p>
             </rich>

</xml_diff>